<commit_message>
Release the row heights again
Forty rows across the course inventory and music education sheets carried a
fixed height and no longer sized to their content. The header rows keep
their 30-point height.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -6465,7 +6465,7 @@
       <c r="T9" s="4"/>
       <c r="U9" s="2"/>
     </row>
-    <row r="10" spans="2:21" ht="126" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
         <v>79</v>
       </c>
@@ -6517,7 +6517,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="2:21" ht="224" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
         <v>88</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="12" spans="2:21" ht="182" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
         <v>97</v>
       </c>
@@ -6619,7 +6619,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="13" spans="2:21" ht="238" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>104</v>
       </c>
@@ -6671,7 +6671,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="2:21" ht="196" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
         <v>110</v>
       </c>
@@ -6719,7 +6719,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="2:21" ht="238" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
         <v>117</v>
       </c>
@@ -6865,7 +6865,7 @@
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
     </row>
-    <row r="18" spans="1:21" ht="182" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B18" s="3" t="s">
         <v>141</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="210" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
         <v>151</v>
       </c>
@@ -6971,7 +6971,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="238" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B20" s="3" t="s">
         <v>158</v>
       </c>
@@ -7067,7 +7067,7 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
     </row>
-    <row r="22" spans="1:21" ht="196" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B22" s="3" t="s">
         <v>169</v>
       </c>
@@ -7121,7 +7121,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="196" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B23" s="3" t="s">
         <v>181</v>
       </c>
@@ -7383,7 +7383,7 @@
       <c r="T27" s="2"/>
       <c r="U27" s="2"/>
     </row>
-    <row r="28" spans="1:21" ht="266" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B28" s="3" t="s">
         <v>214</v>
       </c>
@@ -7483,7 +7483,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="126" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
         <v>232</v>
       </c>
@@ -7532,7 +7532,7 @@
       </c>
       <c r="U30" s="8"/>
     </row>
-    <row r="31" spans="1:21" ht="126" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>232</v>
       </c>
@@ -7625,7 +7625,7 @@
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
     </row>
-    <row r="33" spans="1:21" ht="84" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33" s="6"/>
       <c r="B33" s="3" t="s">
         <v>250</v>
@@ -7674,7 +7674,7 @@
       </c>
       <c r="U33" s="3"/>
     </row>
-    <row r="34" spans="1:21" ht="70" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B34" s="3" t="s">
         <v>257</v>
       </c>
@@ -7722,7 +7722,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="84" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
         <v>232</v>
       </c>
@@ -7817,7 +7817,7 @@
       <c r="T36" s="4"/>
       <c r="U36" s="2"/>
     </row>
-    <row r="37" spans="1:21" ht="293" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B37" s="3" t="s">
         <v>277</v>
       </c>
@@ -7909,7 +7909,7 @@
       <c r="T38" s="2"/>
       <c r="U38" s="2"/>
     </row>
-    <row r="39" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B39" s="2" t="s">
         <v>288</v>
       </c>
@@ -7999,7 +7999,7 @@
       <c r="T40" s="2"/>
       <c r="U40" s="2"/>
     </row>
-    <row r="41" spans="1:21" ht="210" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B41" s="3" t="s">
         <v>297</v>
       </c>
@@ -8053,7 +8053,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="210" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B42" s="3" t="s">
         <v>304</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="43" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B43" s="2" t="s">
         <v>307</v>
       </c>
@@ -8153,7 +8153,7 @@
       <c r="T43" s="2"/>
       <c r="U43" s="2"/>
     </row>
-    <row r="44" spans="1:21" ht="42" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B44" s="2" t="s">
         <v>313</v>
       </c>
@@ -8247,7 +8247,7 @@
       <c r="T45" s="4"/>
       <c r="U45" s="4"/>
     </row>
-    <row r="46" spans="1:21" ht="196" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>232</v>
       </c>
@@ -8352,7 +8352,7 @@
       </c>
       <c r="U47" s="2"/>
     </row>
-    <row r="48" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B48" s="2" t="s">
         <v>343</v>
       </c>
@@ -8396,7 +8396,7 @@
       <c r="T48" s="2"/>
       <c r="U48" s="2"/>
     </row>
-    <row r="49" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B49" s="2" t="s">
         <v>350</v>
       </c>
@@ -8485,7 +8485,7 @@
       <c r="T50" s="2"/>
       <c r="U50" s="2"/>
     </row>
-    <row r="51" spans="1:21" ht="140" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B51" s="3" t="s">
         <v>357</v>
       </c>
@@ -8573,7 +8573,7 @@
       <c r="T52" s="2"/>
       <c r="U52" s="2"/>
     </row>
-    <row r="53" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B53" s="2" t="s">
         <v>365</v>
       </c>
@@ -8617,7 +8617,7 @@
       <c r="T53" s="2"/>
       <c r="U53" s="2"/>
     </row>
-    <row r="54" spans="1:21" ht="28" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B54" s="2" t="s">
         <v>370</v>
       </c>
@@ -8891,7 +8891,7 @@
       <c r="T59" s="4"/>
       <c r="U59" s="2"/>
     </row>
-    <row r="60" spans="1:21" ht="140" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B60" s="3" t="s">
         <v>401</v>
       </c>
@@ -8943,7 +8943,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="168" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B61" s="3" t="s">
         <v>409</v>
       </c>
@@ -8995,7 +8995,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="70" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B62" s="8" t="s">
         <v>416</v>
       </c>
@@ -9181,7 +9181,7 @@
       <c r="T65" s="4"/>
       <c r="U65" s="4"/>
     </row>
-    <row r="66" spans="1:21" ht="84" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
         <v>232</v>
       </c>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="U66" s="13"/>
     </row>
-    <row r="67" spans="1:21" ht="98" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
         <v>232</v>
       </c>
@@ -9283,7 +9283,7 @@
       </c>
       <c r="U67" s="12"/>
     </row>
-    <row r="68" spans="1:21" ht="84" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
         <v>232</v>
       </c>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="U68" s="3"/>
     </row>
-    <row r="69" spans="1:21" ht="70" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
         <v>232</v>
       </c>
@@ -9385,7 +9385,7 @@
       </c>
       <c r="U69" s="8"/>
     </row>
-    <row r="70" spans="1:21" ht="196" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
         <v>232</v>
       </c>
@@ -9436,7 +9436,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="71" spans="1:21" ht="84" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
         <v>232</v>
       </c>
@@ -12773,7 +12773,7 @@
       </c>
       <c r="T10" s="2"/>
     </row>
-    <row r="11" spans="1:20" ht="126" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>749</v>
       </c>
@@ -12967,7 +12967,7 @@
       </c>
       <c r="T14" s="2"/>
     </row>
-    <row r="15" spans="1:20" ht="126" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>769</v>
       </c>

</xml_diff>

<commit_message>
Drop the prerequisite from the MUS 604 revision
MUS 604 carries no prerequisite. The finding and the proposed prerequisite
are removed, leaving the title, description, and learning outcomes.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -6095,24 +6095,6 @@
             </rPr>
             <t>revise the learning outcomes</t>
           </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-no prerequisite published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>prerequisite: graduate standing in music, or department consent</t>
-          </r>
         </is>
       </c>
       <c r="T51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Repair the MUS 604 row
The revision was written one column to the left, overwriting the last
proposal date and putting the proposed content in the technical findings.
The date is restored to 2024-01-31, the three findings sit in
findings_technical, the proposed title, description, and outcomes in
findings_content, and the row is wrapped again.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -5979,58 +5979,58 @@
       <c r="U50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>MUS 604</t>
         </is>
       </c>
-      <c r="C51" s="19" t="inlineStr">
+      <c r="C51" s="11" t="inlineStr">
         <is>
           <t>Sounding Justice: Unveiling the Ecological and Social Dimensions of Music</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Music: Graduate Studies</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>C05 2u</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Explore the transformative nexus of music, environment, and social justice in “Sounding Justice.” Dive into critical analyses, ethical reflections, and applied projects to harness the power of music for positive change.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
-      <c r="J51" s="2" t="n"/>
-      <c r="K51" s="2" t="n"/>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="H51" s="3" t="n"/>
+      <c r="I51" s="3" t="n"/>
+      <c r="J51" s="3" t="n"/>
+      <c r="K51" s="3" t="n"/>
+      <c r="L51" s="3" t="inlineStr">
         <is>
           <t>A-F grading only.</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr">
+      <c r="M51" s="3" t="inlineStr">
         <is>
           <t>On-ground.</t>
         </is>
       </c>
-      <c r="N51" s="2" t="inlineStr">
+      <c r="N51" s="3" t="inlineStr">
         <is>
           <t>Spring Alternate Years</t>
         </is>
       </c>
-      <c r="O51" s="2" t="n"/>
-      <c r="P51" s="2" t="n"/>
-      <c r="Q51" s="2" t="inlineStr">
+      <c r="O51" s="3" t="n"/>
+      <c r="P51" s="3" t="n"/>
+      <c r="Q51" s="3" t="inlineStr">
         <is>
           <t>1. Demonstrate a comprehensive understanding of the intricate relationships between music, the environment, and social justice.
 2. Develop critical analytical skills to assess the impact of music on environmental sustainability and its role in advocating for social change.
@@ -6039,8 +6039,13 @@
 5. Enhance communication proficiency in articulating the relationships between music, the environment, and social justice, both in written and oral formats.</t>
         </is>
       </c>
-      <c r="R51" s="2" t="n"/>
-      <c r="S51" s="2" t="inlineStr">
+      <c r="R51" s="3" t="n"/>
+      <c r="S51" s="3" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="T51" s="3" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6097,7 +6102,7 @@
           </r>
         </is>
       </c>
-      <c r="T51" s="2" t="inlineStr">
+      <c r="U51" s="3" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6157,7 +6162,6 @@
           </r>
         </is>
       </c>
-      <c r="U51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Correct the MUS 324 outcome columns
The four course learning outcomes go in learning_outcomes and the three
Diversity Overlay outcomes in ge_outcomes, matching the 2026-2027 catalog.
The finding is removed.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4292,38 +4292,25 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
+          <t>1) Identify and speak about a range of American musical styles, from the 17th to the 21st centuries;
+2) Correctly employ a range of general and specialized terms relating to music;
+3) Describe the relationship between music and culture and the role music has played in the history of the United States;
+4) Research a topic of your choice in American music and communicate your discoveries through writing and oral presentation.</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
           <t>1. Describe the histories, experiences or views of one or more cultural groups.
 2. Analyze the overlap or intersection of social identities of oneself and/or other cultural groups (e.g., culture, gender, class, sexuality, religion, disability, immigration status, and/or age).
 3. Examine the impact of their own identity on their experiences with and/or views of other cultural groups.</t>
         </is>
       </c>
-      <c r="R33" s="3" t="n"/>
       <c r="S33" s="3" t="inlineStr">
         <is>
           <t>2020-10-06</t>
         </is>
       </c>
-      <c r="T33" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">the three Diversity Overlay outcomes sit in the course learning outcomes, and no course outcomes are published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add course learning outcomes and hold the overlay outcomes as breadth outcomes</t>
-          </r>
-        </is>
-      </c>
+      <c r="T33" s="5" t="n"/>
       <c r="U33" s="3" t="n"/>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Record the MUS 324 instructional method revision
The course is taught on-ground where the record permits hybrid or
online-asynchronous only. The finding sets the methods to on-ground or
hybrid.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4310,7 +4310,27 @@
           <t>2020-10-06</t>
         </is>
       </c>
-      <c r="T33" s="5" t="n"/>
+      <c r="T33" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">instructional methods are hybrid or online-asynchronous, and the course is taught on-ground
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the instructional methods to on-ground or hybrid</t>
+          </r>
+        </is>
+      </c>
       <c r="U33" s="3" t="n"/>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Add the MUS 326 revision
The findings cover the missing learning outcomes, the instructional methods
field holding the course description, and the missing breadth designation.
The content column carries six proposed learning outcomes and the three
Diversity Overlay outcomes.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4415,6 +4415,42 @@
             </rPr>
             <t>add learning outcomes</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+instructional methods field holds the course description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the instructional methods to on-ground, hybrid, online-synchronous, and online-asynchronous</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no breadth designation
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>add the Diversity Overlay</t>
+          </r>
         </is>
       </c>
       <c r="U34" s="5" t="inlineStr">
@@ -4424,17 +4460,42 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no outcomes published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>to be drafted by area faculty</t>
+            <t xml:space="preserve">learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1) Identify and describe the musical traditions, genres, and instruments studied in the semester’s topic, and the communities they belong to;
+2) Analyze how music functions in the religious, political, and social life of those communities, and how identities such as ethnicity, class, gender, and generation intersect in it;
+3) Evaluate the effects of colonization, migration, and commerce on the traditions studied;
+4) Listen critically across unfamiliar repertoires, describing rhythm, melody, texture, and performance practice in appropriate terms;
+5) Examine their own position as listeners in relation to the traditions studied;
+6) Communicate about the semester’s topic in written and oral form, using appropriate vocabulary and critical frameworks.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+breadth outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Describe the histories, experiences or views of one or more cultural groups.
+2. Analyze the overlap or intersection of social identities of oneself and/or other cultural groups (e.g., culture, gender, class, sexuality, religion, disability, immigration status, and/or age).
+3. Examine the impact of their own identity on their experiences with and/or views of other cultural groups.</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Revise the MUS 326 catalog description
The description names the overlay work the course does: traditions in their
religious, political, and social contexts, intersecting identities, and the
student's own position as a listener.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4403,7 +4403,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">no learning outcomes published
+            <t xml:space="preserve">description does not carry the Diversity Overlay outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no learning outcomes published
 </t>
           </r>
           <r>
@@ -4460,7 +4478,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">learning outcomes
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>A rotating-topics course on the music of one world region or diaspora, studied in its religious, political, and social contexts. Students examine how identities intersect in the traditions studied and their own position as listeners. Topics vary by semester.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+learning outcomes
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
Record the current MUS 326 outcomes and revise the proposal
The five outcomes on record go in learning_outcomes. The finding revises
them rather than adding them, and the seven proposed outcomes keep all five
and add the intersecting-identities and own-position work the overlay
requires.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4389,7 +4389,16 @@
       </c>
       <c r="O34" s="3" t="n"/>
       <c r="P34" s="3" t="n"/>
-      <c r="Q34" s="3" t="n"/>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>Because the content of Topics in Global Music changes with each offering, specific goals will vary depending on the topic. However, all versions of this course share core objectives: By the end of the semester, students will:
+• Develop an understanding of the cultural, historical, and stylistic contexts of global musical traditions relevant to the chosen topic.
+• Strengthen skills of listening, analysis, and critical interpretation across diverse musical practices.
+• Engage with primary and secondary sources, including recordings, scholarship, and where possible live or virtual performances, to form informed perspectives.
+• Communicate ideas effectively in written, oral, or creative formats appropriate to the study of music in global contexts.
+• Reflect on how the study of a specialized topic broadens, complicates, or challenges conventional narratives of music history and culture worldwide.</t>
+        </is>
+      </c>
       <c r="R34" s="3" t="n"/>
       <c r="S34" s="3" t="inlineStr">
         <is>
@@ -4421,17 +4430,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-no learning outcomes published
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>add learning outcomes</t>
+learning outcomes do not reach Diversity Overlay outcomes 2 and 3, and open with develop, strengthen, engage, and reflect
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
           </r>
           <r>
             <rPr>
@@ -4510,8 +4519,9 @@
 2) Analyze how music functions in the religious, political, and social life of those communities, and how identities such as ethnicity, class, gender, and generation intersect in it;
 3) Evaluate the effects of colonization, migration, and commerce on the traditions studied;
 4) Listen critically across unfamiliar repertoires, describing rhythm, melody, texture, and performance practice in appropriate terms;
-5) Examine their own position as listeners in relation to the traditions studied;
-6) Communicate about the semester’s topic in written and oral form, using appropriate vocabulary and critical frameworks.</t>
+5) Work with recordings, scholarship, and live or virtual performance to form informed positions on the semester’s topic;
+6) Examine their own position as listeners in relation to the traditions studied, and how the topic complicates the accounts of music history they arrived with;
+7) Communicate about the semester’s topic in written, oral, and creative formats, using appropriate vocabulary and critical frameworks.</t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Tighten the MUS 326 description and outcomes
Six outcomes, each naming an observable product and the evidence it rests
on, and a description that states the overlay work in 39 words.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4497,7 +4497,7 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>A rotating-topics course on the music of one world region or diaspora, studied in its religious, political, and social contexts. Students examine how identities intersect in the traditions studied and their own position as listeners. Topics vary by semester.</t>
+            <t>A rotating-topics course on the music of one world region or diaspora. Students study a repertoire in its religious, political, and social contexts, analyze how identities intersect in it, and account for their own listening. Topics vary by semester.</t>
           </r>
           <r>
             <rPr>
@@ -4515,13 +4515,12 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1) Identify and describe the musical traditions, genres, and instruments studied in the semester’s topic, and the communities they belong to;
-2) Analyze how music functions in the religious, political, and social life of those communities, and how identities such as ethnicity, class, gender, and generation intersect in it;
-3) Evaluate the effects of colonization, migration, and commerce on the traditions studied;
-4) Listen critically across unfamiliar repertoires, describing rhythm, melody, texture, and performance practice in appropriate terms;
-5) Work with recordings, scholarship, and live or virtual performance to form informed positions on the semester’s topic;
-6) Examine their own position as listeners in relation to the traditions studied, and how the topic complicates the accounts of music history they arrived with;
-7) Communicate about the semester’s topic in written, oral, and creative formats, using appropriate vocabulary and critical frameworks.</t>
+            <t>1) Identify by ear and describe in writing the principal genres, instruments, and performance practices of the semester’s region or diaspora, naming the communities that carry them;
+2) Explain how a specific repertoire functions in the religious, political, or social life of the community that made it, citing recordings and scholarship;
+3) Analyze how ethnicity, class, gender, generation, religion, or migration status intersect in a specific musical practice, and what that intersection means for who performs it and who hears it;
+4) Trace what colonization, migration, or commercial circulation changed in a tradition, using recordings and scholarship as evidence;
+5) Account in writing for their own position as a listener: what they expected, what they heard, and how their own background shaped the difference;
+6) Present findings on a tradition in written and spoken form for a non-specialist audience, using the vocabulary and citation conventions of the field.</t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Mark MUS 326 done
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -190,6 +190,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4334,6 +4337,11 @@
       <c r="U33" s="3" t="n"/>
     </row>
     <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
           <t>MUS 326</t>

</xml_diff>

<commit_message>
Mark MUS 324 and MUS 604 done
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4237,7 +4237,11 @@
       <c r="U32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
           <t>MUS 324</t>
@@ -6100,6 +6104,11 @@
       <c r="U50" s="2" t="n"/>
     </row>
     <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
           <t>MUS 604</t>

</xml_diff>

<commit_message>
Flag the offering patterns in the theory and musicianship sequence
Six courses publish an offering pattern the guide contradicts: MUS 112,
116, 211, and 215 are Variable Intermittently, and MUS 312 and 410 are
alternate years, where the guide runs each of them annually in a fixed
semester.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1594,6 +1594,24 @@
             </rPr>
             <t>remove the strongly recommended preparation</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+offered Variable Intermittently where the guide runs Theory II every fall
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Fall</t>
+          </r>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
@@ -1913,6 +1931,24 @@
               <sz val="10"/>
             </rPr>
             <t>corequisite: MUS 112 and MUS 119, or equivalent, or department consent</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+offered Variable Intermittently where the guide runs Aural Skills II every fall
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Fall</t>
           </r>
         </is>
       </c>
@@ -2557,6 +2593,24 @@
             </rPr>
             <t>remove the strongly recommended preparation</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+offered Variable Intermittently where the guide runs Theory III every spring
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Spring</t>
+          </r>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
@@ -2709,6 +2763,24 @@
               <sz val="10"/>
             </rPr>
             <t>corequisite: MUS 211 and MUS 218, or equivalent, or department consent</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+offered Variable Intermittently where the guide runs Aural Skills III every spring
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Spring</t>
           </r>
         </is>
       </c>
@@ -3851,6 +3923,24 @@
             </rPr>
             <t>prerequisite: MUS 211, MUS 215, and MUS 218, or successful Theory and Musicianship Placement Exam, or department consent</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+offered Fall Alternate Years where the guide runs Form and Analysis every fall
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Fall</t>
+          </r>
         </is>
       </c>
       <c r="U28" s="5" t="inlineStr">
@@ -4828,6 +4918,24 @@
               <sz val="10"/>
             </rPr>
             <t>prerequisite: MUS 312, or equivalent, or department consent</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+offered Spring Alternate Years where the guide runs the course every spring
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Spring</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Flag the coaching corequisites and offering patterns
The four undergraduate coaching courses name applied study ranges that run
past the last course in each series and do not separate voice from
instrument. MUS 660A and 660B publish no offering pattern.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3204,6 +3204,24 @@
             </rPr>
             <t>revise the learning outcomes</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+corequisite names the MUS 261-269 series, which ends at MUS 266, and admits applied study on any instrument
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>corequisite: MUS 262 or MUS 262G, or department consent</t>
+          </r>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
@@ -3399,6 +3417,24 @@
               <sz val="10"/>
             </rPr>
             <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+corequisite names the MUS 261-269 series, which ends at MUS 266, and admits applied study in voice
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>corequisite: one of MUS 261, 261G, 263, 263G, 264, 265, 266, or department consent</t>
           </r>
         </is>
       </c>
@@ -5306,6 +5342,24 @@
             </rPr>
             <t>revise the learning outcomes</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+corequisite names the MUS 461-469 series, which ends at MUS 468, and admits applied study on any instrument
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>corequisite: MUS 462, or department consent</t>
+          </r>
         </is>
       </c>
       <c r="U41" s="5" t="inlineStr">
@@ -5465,6 +5519,24 @@
               <sz val="10"/>
             </rPr>
             <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+corequisite names the MUS 461-469 series, which ends at MUS 468, and admits applied study in voice
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>corequisite: one of MUS 461, 461A, 463, 463A, 464, 464A, 465, 465A, 466, 466A, 467, 467A, 468, or department consent</t>
           </r>
         </is>
       </c>
@@ -7140,6 +7212,24 @@
             </rPr>
             <t>revise the description</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no offering pattern published
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Fall and Spring</t>
+          </r>
         </is>
       </c>
       <c r="U60" s="3" t="inlineStr">
@@ -7309,6 +7399,24 @@
               <sz val="10"/>
             </rPr>
             <t>revise the description</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no offering pattern published
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Fall and Spring</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Match the graduate coaching corequisites to the undergraduate pattern
MUS 660A takes MUS 662, or department consent. MUS 660B takes one of the
graduate instrumental applied courses, or department consent, with the
range ending at MUS 668. Department consent stays as the prerequisite on
all six coaching courses.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -7182,17 +7182,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-prerequisite of department consent, absent on most graduate applied courses
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>remove or apply it across the series</t>
+corequisite carries no consent path
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>corequisite: MUS 662, or department consent</t>
           </r>
           <r>
             <rPr>
@@ -7352,35 +7352,17 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-requires MUS 669, renumbered or discontinued
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>end the range at MUS 668</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-prerequisite of department consent, absent on most graduate applied courses
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>remove or apply it across the series</t>
+corequisite requires MUS 669, which does not exist, and carries no consent path
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>corequisite: one of MUS 661, 661A, 663, 663A, 664, 664A, 665, 665A, 666, 666A, 667, 668, or department consent</t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
Remove the prerequisite from the coaching series
The consent path now sits in the corequisite on all six courses, so the
standing prerequisite of department consent is dropped.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3222,6 +3222,24 @@
             </rPr>
             <t>corequisite: MUS 262 or MUS 262G, or department consent</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent duplicates the consent path in the corequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the prerequisite</t>
+          </r>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
@@ -3435,6 +3453,24 @@
               <sz val="10"/>
             </rPr>
             <t>corequisite: one of MUS 261, 261G, 263, 263G, 264, 265, 266, or department consent</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent duplicates the consent path in the corequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the prerequisite</t>
           </r>
         </is>
       </c>
@@ -5360,6 +5396,24 @@
             </rPr>
             <t>corequisite: MUS 462, or department consent</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent duplicates the consent path in the corequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the prerequisite</t>
+          </r>
         </is>
       </c>
       <c r="U41" s="5" t="inlineStr">
@@ -5537,6 +5591,24 @@
               <sz val="10"/>
             </rPr>
             <t>corequisite: one of MUS 461, 461A, 463, 463A, 464, 464A, 465, 465A, 466, 466A, 467, 467A, 468, or department consent</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent duplicates the consent path in the corequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the prerequisite</t>
           </r>
         </is>
       </c>
@@ -7230,6 +7302,24 @@
             </rPr>
             <t>set the offering pattern to Fall and Spring</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent duplicates the consent path in the corequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the prerequisite</t>
+          </r>
         </is>
       </c>
       <c r="U60" s="3" t="inlineStr">
@@ -7399,6 +7489,24 @@
               <sz val="10"/>
             </rPr>
             <t>set the offering pattern to Fall and Spring</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent duplicates the consent path in the corequisite
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the prerequisite</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Correct the coaching unit finding
The handbook states no unit requirement for a recital semester. MUS 281 and
282 are fixed at 1 unit where the rest of the series publishes 1-2. MUS
660A and 660B carry a note that the Graduate Student Handbook calls them
2-unit courses.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3138,7 +3138,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
+            <t xml:space="preserve">fixed at 1 unit where the rest of the coaching series publishes 1–2
 </t>
           </r>
           <r>
@@ -3370,7 +3370,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">fixed at 1 unit, so a recitalist cannot enroll in the 2 units the handbook requires in the recital semester
+            <t xml:space="preserve">fixed at 1 unit where the rest of the coaching series publishes 1–2
 </t>
           </r>
           <r>
@@ -7320,6 +7320,24 @@
             </rPr>
             <t>remove the prerequisite</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+publishes 1–2 units where the Graduate Student Handbook calls it a 2-unit course
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>reconcile the handbook with the record</t>
+          </r>
         </is>
       </c>
       <c r="U60" s="3" t="inlineStr">
@@ -7507,6 +7525,24 @@
               <sz val="10"/>
             </rPr>
             <t>remove the prerequisite</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+publishes 1–2 units where the Graduate Student Handbook calls it a 2-unit course
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>reconcile the handbook with the record</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
Mark MUS 281 done
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3054,6 +3054,11 @@
       <c r="U21" s="18" t="n"/>
     </row>
     <row r="22" s="17">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
           <t>MUS 281</t>

</xml_diff>

<commit_message>
clear the MUS 360A grading finding
MUS 360A publishes the chamber ensemble grading value without a
closing period. The value matches the norm and needs no revision.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -12971,27 +12971,7 @@
           <t>2025-09-14</t>
         </is>
       </c>
-      <c r="S7" s="19" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">grading A-F or CR/NC (student choice) where the chamber ensemble norm is A-F or CR/NC (student choice)
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set grading to A-F or CR/NC (student choice) or confirm the difference is intended</t>
-          </r>
-        </is>
-      </c>
+      <c r="S7" s="19"/>
       <c r="T7" s="18" t="n"/>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
set MUS 664A to 1-2 units in the inventory
Replace the conflicting unit findings on MUS 664A with one change:
publish 1-2 units, matching the record and the graduate applied series.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -11783,25 +11783,7 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1 where the record holds 1-2
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>set units to 1</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-units publish as 1 where the other graduate applied courses publish 1–2
+            <t xml:space="preserve">units publish as 1 where the record holds 1–2 and the other graduate applied courses publish 1–2
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
add the C36 1-2u classification finding to graduate applied study
MUS 661 through MUS 668, including the lettered courses, record C36 1u
and publish 1-2 units. Each now carries the classification change set
on MUS 660A and MUS 660B.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -11266,7 +11266,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent, absent on most graduate applied courses
 </t>
           </r>
           <r>
@@ -11363,7 +11381,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent, absent on most graduate applied courses
 </t>
           </r>
           <r>
@@ -11456,7 +11492,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">description runs to 41 words, over the 40-word limit
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+description runs to 41 words, over the 40-word limit
 </t>
           </r>
           <r>
@@ -11558,7 +11612,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S28" s="18" t="n"/>
+      <c r="S28" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T28" s="18" t="n"/>
     </row>
     <row r="29">
@@ -11631,7 +11705,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S29" s="18" t="n"/>
+      <c r="S29" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T29" s="18" t="n"/>
     </row>
     <row r="30">
@@ -11704,7 +11798,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S30" s="18" t="n"/>
+      <c r="S30" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T30" s="18" t="n"/>
     </row>
     <row r="31">
@@ -11783,7 +11897,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">units publish as 1 where the record holds 1–2 and the other graduate applied courses publish 1–2
+            <t xml:space="preserve">classification records 1 unit where the record holds 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+units publish as 1 where the record holds 1–2 and the other graduate applied courses publish 1–2
 </t>
           </r>
           <r>
@@ -11869,7 +12001,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S32" s="18" t="n"/>
+      <c r="S32" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T32" s="18" t="n"/>
     </row>
     <row r="33">
@@ -11942,7 +12094,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S33" s="18" t="n"/>
+      <c r="S33" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T33" s="18" t="n"/>
     </row>
     <row r="34">
@@ -12015,7 +12187,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S34" s="18" t="n"/>
+      <c r="S34" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T34" s="18" t="n"/>
     </row>
     <row r="35">
@@ -12098,7 +12290,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">prerequisite of department consent, absent on most graduate applied courses
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+prerequisite of department consent, absent on most graduate applied courses
 </t>
           </r>
           <r>
@@ -12184,7 +12394,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S36" s="18" t="n"/>
+      <c r="S36" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T36" s="18" t="n"/>
     </row>
     <row r="37">
@@ -12257,7 +12487,27 @@
           <t>2024-01-31</t>
         </is>
       </c>
-      <c r="S37" s="18" t="n"/>
+      <c r="S37" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">classification records 1 unit where the course publishes 1–2
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the classification to C36 1-2u</t>
+          </r>
+        </is>
+      </c>
       <c r="T37" s="18" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mark MUS 282, 481, and 482 done
The undergraduate coaching series proposals are launched in Curriculog.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3291,6 +3291,11 @@
       </c>
     </row>
     <row r="23" s="17">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
           <t>MUS 282</t>
@@ -5269,6 +5274,11 @@
       <c r="U40" s="18" t="n"/>
     </row>
     <row r="41" s="17">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
           <t>MUS 481</t>
@@ -5465,6 +5475,11 @@
       </c>
     </row>
     <row r="42" s="17">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
           <t>MUS 482</t>

</xml_diff>

<commit_message>
add revised learning outcomes for MUS 660A and 660B
Both rows gain a learning outcomes finding and the revised outcomes.
The handbook units finding is removed; the handbook now reads 1-2 units.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -7310,6 +7310,24 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
+learning outcomes are written as development goals and name no assessable product
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
 no offering pattern published
 </t>
           </r>
@@ -7340,44 +7358,48 @@
             </rPr>
             <t>remove the prerequisite</t>
           </r>
+        </is>
+      </c>
+      <c r="U60" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Individual vocal coaching with a collaborative pianist for graduate students, in preparation for the graduate recital. Coaching times arranged according to the expectations in the Graduate Student Handbook.</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-publishes 1–2 units where the Graduate Student Handbook calls it a 2-unit course
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reconcile the handbook with the record</t>
-          </r>
-        </is>
-      </c>
-      <c r="U60" s="3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Individual vocal coaching with a collaborative pianist for graduate students, in preparation for the graduate recital. Coaching times arranged according to the expectations in the Graduate Student Handbook.</t>
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Build a graduate recital program with a collaborative pianist, taking responsibility for repertoire, order, and pacing.
+2. Apply diction, translation, poetic interpretation, and character development across repertoire in more than one language.
+3. Lead rehearsals with a collaborative pianist, setting the interpretive decisions and revising them across the preparation.
+4. Write program notes that document the sources, style, and interpretive decisions of the program.
+5. Perform a program that meets the graduate recital requirements in the Graduate Student Handbook.</t>
           </r>
         </is>
       </c>
@@ -7516,6 +7538,24 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
+learning outcomes are written as development goals and name no assessable product
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>revise the learning outcomes</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
 no offering pattern published
 </t>
           </r>
@@ -7546,44 +7586,48 @@
             </rPr>
             <t>remove the prerequisite</t>
           </r>
+        </is>
+      </c>
+      <c r="U61" s="3" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Individual instrumental coaching with a collaborative pianist for graduate students, in preparation for the graduate recital. Coaching times arranged according to the expectations in the Graduate Student Handbook.</t>
+          </r>
           <r>
             <rPr>
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-publishes 1–2 units where the Graduate Student Handbook calls it a 2-unit course
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>reconcile the handbook with the record</t>
-          </r>
-        </is>
-      </c>
-      <c r="U61" s="3" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Individual instrumental coaching with a collaborative pianist for graduate students, in preparation for the graduate recital. Coaching times arranged according to the expectations in the Graduate Student Handbook.</t>
+learning outcomes
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. Build a graduate recital program with a collaborative pianist, taking responsibility for repertoire, order, and pacing.
+2. Apply articulation, phrasing, intonation, and stylistic decisions drawn from performance practice across repertoire from more than one period.
+3. Lead rehearsals with a collaborative pianist, setting the interpretive decisions and revising them across the preparation.
+4. Write program notes that document the sources, style, and interpretive decisions of the program.
+5. Perform a program that meets the graduate recital requirements in the Graduate Student Handbook.</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
mark MUS 660A and 660B done
The graduate coaching proposals are launched in Curriculog.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -7176,6 +7176,11 @@
       <c r="U59" s="18" t="n"/>
     </row>
     <row r="60" s="17">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
           <t>MUS 660A</t>
@@ -7405,6 +7410,11 @@
       </c>
     </row>
     <row r="61" s="17">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
           <t>MUS 660B</t>

</xml_diff>

<commit_message>
clear the MUS 317 findings
MUS 317 is not being revised.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -4137,48 +4137,8 @@
           <t>2023-09-15</t>
         </is>
       </c>
-      <c r="T29" s="19" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description runs to 42 words, over the 40-word limit
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>shorten to 40 words or fewer</t>
-          </r>
-        </is>
-      </c>
-      <c r="U29" s="19" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">description
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <b val="1"/>
-              <color rgb="FFB03A2E"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Development of soloing techniques idiomatic to the bebop and post-bop traditions. Includes jazz theory, analysis and performance of transcriptions by bebop and post-bop masters, and in-class application of the devices used in modern jazz improvisation.</t>
-          </r>
-        </is>
-      </c>
+      <c r="T29" s="19"/>
+      <c r="U29" s="19"/>
     </row>
     <row r="30" s="17">
       <c r="A30" s="16" t="inlineStr">

</xml_diff>

<commit_message>
defer MUS 600 and 622, unwrap rows not in progress
MUS 600 and MUS 622 carry status D. MUS 317, 600, and 622 have wrap
text off across the row. Adds a status cell style without wrap.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -205,6 +205,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4071,7 +4074,7 @@
           <t>MUS 317</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Improvisation Techniques</t>
         </is>
@@ -6050,12 +6053,17 @@
       </c>
     </row>
     <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
           <t>MUS 600</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C47" s="18" t="inlineStr">
         <is>
           <t>Seminar in Research Methodology</t>
         </is>
@@ -6751,12 +6759,17 @@
       <c r="U54" s="18" t="n"/>
     </row>
     <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
           <t>MUS 622</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C55" s="18" t="inlineStr">
         <is>
           <t>Seminar in Asian Music and Culture</t>
         </is>

</xml_diff>

<commit_message>
mark MUS 312 and 410 done
The proposals are launched in Curriculog. The MUS 312 classification
item is removed from the catalog-audit open items.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -3884,6 +3884,11 @@
       <c r="U27" s="18" t="n"/>
     </row>
     <row r="28" s="17">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
           <t>MUS 312</t>
@@ -4862,6 +4867,11 @@
       <c r="U36" s="18" t="n"/>
     </row>
     <row r="37" s="17">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
           <t>MUS 410</t>

</xml_diff>

<commit_message>
change the deferred status code from D to DFR
MUS 600 and MUS 622 now read DFR.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -6065,7 +6065,7 @@
     <row r="47">
       <c r="A47" s="22" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DFR</t>
         </is>
       </c>
       <c r="B47" s="18" t="inlineStr">
@@ -6771,7 +6771,7 @@
     <row r="55">
       <c r="A55" s="22" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DFR</t>
         </is>
       </c>
       <c r="B55" s="18" t="inlineStr">

</xml_diff>

<commit_message>
put proposed outcomes on numbered lines
The revised outcomes for MUS 111, 112, 115, 116, 118, 119, 211, 215,
218, 312, and 410 now list one outcome per line.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1463,7 +1463,11 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Read, write, and analyze the fundamental materials of tonal music using correct terminology and nomenclature. 2. Construct and identify all triad and seventh chord types in root position and inversion. 3. Write four-part (SATB) harmonic progressions using I, V, V⁷, and their inversions, applying basic voice-leading principles. 4. Compose and analyze two-voice counterpoint through fourth species. 5. Apply theoretical concepts at the keyboard and in performance on the student's primary instrument or voice.</t>
+            <t xml:space="preserve">1. Read, write, and analyze the fundamental materials of tonal music using correct terminology and nomenclature.
+2. Construct and identify all triad and seventh chord types in root position and inversion.
+3. Write four-part (SATB) harmonic progressions using I, V, V⁷, and their inversions, applying basic voice-leading principles.
+4. Compose and analyze two-voice counterpoint through fourth species.
+5. Apply theoretical concepts at the keyboard and in performance on the student's primary instrument or voice.</t>
           </r>
         </is>
       </c>
@@ -1652,7 +1656,11 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Write and analyze SATB progressions using the full vocabulary of diatonic harmony, including all diatonic triads and seventh chords. 2. Identify and apply embellishing chords, the cadential 6/4, and other 6/4 chord types in functional context. 3. Recognize and compose diatonic sequences. 4. Analyze tonal works using Roman numerals, figured bass, and functional labels. 5. Apply diatonic harmonic vocabulary at the keyboard and in performance on the student's primary instrument or voice.</t>
+            <t xml:space="preserve">1. Write and analyze SATB progressions using the full vocabulary of diatonic harmony, including all diatonic triads and seventh chords.
+2. Identify and apply embellishing chords, the cadential 6/4, and other 6/4 chord types in functional context.
+3. Recognize and compose diatonic sequences.
+4. Analyze tonal works using Roman numerals, figured bass, and functional labels.
+5. Apply diatonic harmonic vocabulary at the keyboard and in performance on the student's primary instrument or voice.</t>
           </r>
         </is>
       </c>
@@ -1801,7 +1809,10 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Sight-sing diatonic melodies in major keys and simple meters using solfège or scale degrees, with accurate pitch, rhythm, and conducting. 2. Take melodic and rhythmic dictation in simple meters, notating pitch and rhythm accurately, including ties and the dotted beat. 3. Detect and correct errors in performed and notated examples. 4. Read fluently across all fifteen major keys.</t>
+            <t xml:space="preserve">1. Sight-sing diatonic melodies in major keys and simple meters using solfège or scale degrees, with accurate pitch, rhythm, and conducting.
+2. Take melodic and rhythmic dictation in simple meters, notating pitch and rhythm accurately, including ties and the dotted beat.
+3. Detect and correct errors in performed and notated examples.
+4. Read fluently across all fifteen major keys.</t>
           </r>
         </is>
       </c>
@@ -1990,7 +2001,10 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Sight-sing diatonic melodies in minor mode, approached through both relative and parallel major and including chromatic 6 and 7 by modal borrowing, and in compound meters, using solfège or scale degrees. 2. Take melodic and rhythmic dictation extending to triplets and duplets, quadruple division in simple meter, sextuple division in compound meter, and syncopation. 3. Perform lower chromatic neighbors and melodic skips to chord tones as prefix neighbors through the tonic, dominant, and subdominant triads. 4. Sing the dominant seventh chord in melodic context.</t>
+            <t xml:space="preserve">1. Sight-sing diatonic melodies in minor mode, approached through both relative and parallel major and including chromatic 6 and 7 by modal borrowing, and in compound meters, using solfège or scale degrees.
+2. Take melodic and rhythmic dictation extending to triplets and duplets, quadruple division in simple meter, sextuple division in compound meter, and syncopation.
+3. Perform lower chromatic neighbors and melodic skips to chord tones as prefix neighbors through the tonic, dominant, and subdominant triads.
+4. Sing the dominant seventh chord in melodic context.</t>
           </r>
         </is>
       </c>
@@ -2122,7 +2136,11 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Perform major and minor five-finger patterns and their triads in all common keys. 2. Perform all four triad qualities (major, minor, augmented, diminished) in root position. 3. Play major scales in tetrachord position with correct fingering, and use the damper pedal. 4. Harmonize simple melodies using basic diatonic chords. 5. Sight-read short examples in grand staff at a basic level.</t>
+            <t xml:space="preserve">1. Perform major and minor five-finger patterns and their triads in all common keys.
+2. Perform all four triad qualities (major, minor, augmented, diminished) in root position.
+3. Play major scales in tetrachord position with correct fingering, and use the damper pedal.
+4. Harmonize simple melodies using basic diatonic chords.
+5. Sight-read short examples in grand staff at a basic level.</t>
           </r>
         </is>
       </c>
@@ -2275,7 +2293,12 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Perform major and minor scales and arpeggios across Group 1 and Group 2 keys, two octaves. 2. Play triads in all inversions and perform the dominant seventh chord in block and broken patterns. 3. Harmonize short melodies using primary chords (I, IV, V⁷) in major and minor, with idiomatic accompaniment patterns including Alberti and waltz bass. 4. Sing a melody while playing a two-hand accompaniment. 5. Realize basic lead-sheet symbols and Roman numerals at the keyboard. 6. Sight-read in grand staff, hands together, in four-to-eight-bar examples.</t>
+            <t xml:space="preserve">1. Perform major and minor scales and arpeggios across Group 1 and Group 2 keys, two octaves.
+2. Play triads in all inversions and perform the dominant seventh chord in block and broken patterns.
+3. Harmonize short melodies using primary chords (I, IV, V⁷) in major and minor, with idiomatic accompaniment patterns including Alberti and waltz bass.
+4. Sing a melody while playing a two-hand accompaniment.
+5. Realize basic lead-sheet symbols and Roman numerals at the keyboard.
+6. Sight-read in grand staff, hands together, in four-to-eight-bar examples.</t>
           </r>
         </is>
       </c>
@@ -2633,7 +2656,11 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Write and analyze chromatic harmony, including applied dominants, modal mixture, the Neapolitan sixth, augmented sixth chords, and altered chords. 2. Identify and compose modulations to the dominant and to closely related keys. 3. Analyze chromatic sequences and chromatic modulation. 4. Evaluate tonal works combining diatonic and chromatic vocabulary in extended harmonic contexts. 5. Apply chromatic harmonic vocabulary at the keyboard and in performance on the student's primary instrument or voice.</t>
+            <t xml:space="preserve">1. Write and analyze chromatic harmony, including applied dominants, modal mixture, the Neapolitan sixth, augmented sixth chords, and altered chords.
+2. Identify and compose modulations to the dominant and to closely related keys.
+3. Analyze chromatic sequences and chromatic modulation.
+4. Evaluate tonal works combining diatonic and chromatic vocabulary in extended harmonic contexts.
+5. Apply chromatic harmonic vocabulary at the keyboard and in performance on the student's primary instrument or voice.</t>
           </r>
         </is>
       </c>
@@ -2822,7 +2849,10 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Sing and hear harmonically, following harmonic rhythm and cadences. 2. Work in two-voice textures and take bass-line dictation. 3. Identify root-position and first-inversion triads and all four triad qualities by ear, and sing melodic skips through every diatonic triad (leading-tone, supertonic, submediant, and mediant). 4. Handle the dominant seventh chord in harmonic context, with the voice-leading techniques that close the lower-division sequence.</t>
+            <t xml:space="preserve">1. Sing and hear harmonically, following harmonic rhythm and cadences.
+2. Work in two-voice textures and take bass-line dictation.
+3. Identify root-position and first-inversion triads and all four triad qualities by ear, and sing melodic skips through every diatonic triad (leading-tone, supertonic, submediant, and mediant).
+4. Handle the dominant seventh chord in harmonic context, with the voice-leading techniques that close the lower-division sequence.</t>
           </r>
         </is>
       </c>
@@ -2975,7 +3005,12 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Perform major and minor scales and arpeggios across all key groups, and play chromatic, whole-tone, and blues scales. 2. Perform secondary triads (ii, iii, vi) and seventh chords in harmonic context, with correct voice leading. 3. Play melodies and accompaniments in all six church modes. 4. Harmonize melodies using the full diatonic vocabulary including secondary chords. 5. Transpose short examples to other keys and improvise within defined modal and harmonic frameworks. 6. Prepare and perform repertoire from Alfred's Book 1 for peers and instructor.</t>
+            <t xml:space="preserve">1. Perform major and minor scales and arpeggios across all key groups, and play chromatic, whole-tone, and blues scales.
+2. Perform secondary triads (ii, iii, vi) and seventh chords in harmonic context, with correct voice leading.
+3. Play melodies and accompaniments in all six church modes.
+4. Harmonize melodies using the full diatonic vocabulary including secondary chords.
+5. Transpose short examples to other keys and improvise within defined modal and harmonic frameworks.
+6. Prepare and perform repertoire from Alfred's Book 1 for peers and instructor.</t>
           </r>
         </is>
       </c>
@@ -4068,7 +4103,12 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Demonstrate understanding of the forms used in tonal music, including sentence, period, binary, ternary, rondo, and sonata forms. 2. Analyze and evaluate complete tonal works in their technical, aesthetic, and historical contexts, supporting interpretive claims with evidence from the score. 3. Apply the harmonic and contrapuntal knowledge of the lower-division sequence to extended musical works. 4. Identify phrase structure, hypermeter, and formal boundaries both visually and aurally. 5. Construct written analyses using appropriate terminology, Roman numerals, figured bass, and formal labels. 6. Implement the principles and concepts studied in class via performance on the student's major instrument or voice.</t>
+            <t xml:space="preserve">1. Demonstrate understanding of the forms used in tonal music, including sentence, period, binary, ternary, rondo, and sonata forms.
+2. Analyze and evaluate complete tonal works in their technical, aesthetic, and historical contexts, supporting interpretive claims with evidence from the score.
+3. Apply the harmonic and contrapuntal knowledge of the lower-division sequence to extended musical works.
+4. Identify phrase structure, hypermeter, and formal boundaries both visually and aurally.
+5. Construct written analyses using appropriate terminology, Roman numerals, figured bass, and formal labels.
+6. Implement the principles and concepts studied in class via performance on the student's major instrument or voice.</t>
           </r>
         </is>
       </c>
@@ -5029,7 +5069,12 @@
               <color rgb="FFB03A2E"/>
               <sz val="10"/>
             </rPr>
-            <t>1. Demonstrate understanding of the different genres, styles, and techniques of 20th and 21st century art music. 2. Analyze and evaluate post-tonal works in their technical, aesthetic, and historical contexts, supporting interpretive claims with evidence from the score. 3. Construct and manipulate post-tonal pitch collections, including pitch-class sets in normal and prime form, and analyze twelve-tone rows and their transformations. 4. Apply knowledge from earlier theory courses to extended post-tonal and contemporary works. 5. Situate works within the major compositional movements of the 20th and 21st centuries, including serialism, spectralism, minimalism, and extended techniques. 6. Implement the principles and concepts studied in class via performance on the student's area of emphasis.</t>
+            <t xml:space="preserve">1. Demonstrate understanding of the different genres, styles, and techniques of 20th and 21st century art music.
+2. Analyze and evaluate post-tonal works in their technical, aesthetic, and historical contexts, supporting interpretive claims with evidence from the score.
+3. Construct and manipulate post-tonal pitch collections, including pitch-class sets in normal and prime form, and analyze twelve-tone rows and their transformations.
+4. Apply knowledge from earlier theory courses to extended post-tonal and contemporary works.
+5. Situate works within the major compositional movements of the 20th and 21st centuries, including serialism, spectralism, minimalism, and extended techniques.
+6. Implement the principles and concepts studied in class via performance on the student's area of emphasis.</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
add the MUS 111 description finding
The proposed description matches the MUS 111 syllabus.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1453,7 +1453,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes are generic to the sequence and name no level-specific content, where the syllabus outcomes from the musicianship overhaul are current
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The first of three intensive courses that introduce students to the inner workings of European art music of the 18th and 19th centuries. This course covers diatonic harmony, as well as part-writing, voice-leading, and harmonization techniques.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+outcomes are generic to the sequence and name no level-specific content, where the syllabus outcomes from the musicianship overhaul are current
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
add the MUS 211 description finding
The proposed description matches the MUS 211 syllabus.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -2664,7 +2664,25 @@
               <rFont val="Arial"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">outcomes repeat the closing three of MUS 111 and MUS 112 and name no level-specific content, where the syllabus outcomes from the musicianship overhaul are current
+            <t xml:space="preserve">description
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>The last of three intensive courses that introduce students to the inner workings of European art music of the 18th and 19th centuries. This course covers chromatic harmony, tonicization and modulation, and other advanced tonal procedures.</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+outcomes repeat the closing three of MUS 111 and MUS 112 and name no level-specific content, where the syllabus outcomes from the musicianship overhaul are current
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
mark the theory and aural skills tracks done
MUS 111, 112, 211, 115, 116, and 215 are launched in Curriculog.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -1333,6 +1333,11 @@
       <c r="U9" s="18" t="n"/>
     </row>
     <row r="10" s="17">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t>MUS 111</t>
@@ -1491,6 +1496,11 @@
       </c>
     </row>
     <row r="11" s="17">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>MUS 112</t>
@@ -1684,6 +1694,11 @@
       </c>
     </row>
     <row r="12" s="17">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>MUS 115</t>
@@ -1836,6 +1851,11 @@
       </c>
     </row>
     <row r="13" s="17">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>MUS 116</t>
@@ -2487,6 +2507,11 @@
       <c r="U17" s="18" t="n"/>
     </row>
     <row r="18" s="17">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>MUS 211</t>
@@ -2702,6 +2727,11 @@
       </c>
     </row>
     <row r="19" s="17">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>MUS 215</t>

</xml_diff>

<commit_message>
mark the keyboard track done
MUS 118, 119, and 218 are launched in Curriculog.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -2048,6 +2048,11 @@
       </c>
     </row>
     <row r="14" s="17">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>MUS 118</t>
@@ -2184,6 +2189,11 @@
       </c>
     </row>
     <row r="15" s="17">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>MUS 119</t>
@@ -2924,6 +2934,11 @@
       </c>
     </row>
     <row r="20" s="17">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>MUS 218</t>

</xml_diff>

<commit_message>
add the MUS 698 credit restriction and offering findings
The credit restriction is removed and the offering pattern is set to
Fall and Spring, as in MUS 498.
</commit_message>
<xml_diff>
--- a/curriculum/catalog-audit/course-inventory.xlsx
+++ b/curriculum/catalog-audit/course-inventory.xlsx
@@ -8522,6 +8522,42 @@
             </rPr>
             <t>add learning outcomes</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+credit restriction keeps internship units off the degree and is cut off mid-sentence in the catalog
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>remove the credit restriction</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+no offering pattern published
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FFB03A2E"/>
+              <sz val="10"/>
+            </rPr>
+            <t>set the offering pattern to Fall &amp; Spring</t>
+          </r>
         </is>
       </c>
       <c r="U70" s="14" t="inlineStr">

</xml_diff>